<commit_message>
DEA analysis script update - SBM imports results
</commit_message>
<xml_diff>
--- a/DEA_results/SBM_exports_results.xlsx
+++ b/DEA_results/SBM_exports_results.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B173"/>
+  <dimension ref="A1:C173"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,6 +362,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>iso3</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Efficiency</t>
         </is>
       </c>
@@ -372,7 +377,12 @@
           <t>Albania</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="C2">
         <v>0.4123818969882356</v>
       </c>
     </row>
@@ -382,7 +392,12 @@
           <t>Algeria</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DZA</t>
+        </is>
+      </c>
+      <c r="C3">
         <v>0.2113920319811434</v>
       </c>
     </row>
@@ -392,7 +407,12 @@
           <t>Angola</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
@@ -402,7 +422,12 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ARG</t>
+        </is>
+      </c>
+      <c r="C5">
         <v>0.1322574754520223</v>
       </c>
     </row>
@@ -412,7 +437,12 @@
           <t>Armenia</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="C6">
         <v>1</v>
       </c>
     </row>
@@ -422,7 +452,12 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AUS</t>
+        </is>
+      </c>
+      <c r="C7">
         <v>1</v>
       </c>
     </row>
@@ -432,7 +467,12 @@
           <t>Austria</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AUT</t>
+        </is>
+      </c>
+      <c r="C8">
         <v>1</v>
       </c>
     </row>
@@ -442,7 +482,12 @@
           <t>Azerbaijan</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AZE</t>
+        </is>
+      </c>
+      <c r="C9">
         <v>0.4265918044718086</v>
       </c>
     </row>
@@ -452,7 +497,12 @@
           <t>Bahamas</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BHS</t>
+        </is>
+      </c>
+      <c r="C10">
         <v>1</v>
       </c>
     </row>
@@ -462,7 +512,12 @@
           <t>Bahrain</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BHR</t>
+        </is>
+      </c>
+      <c r="C11">
         <v>0.3124411173268752</v>
       </c>
     </row>
@@ -472,7 +527,12 @@
           <t>Bangladesh</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="C12">
         <v>1</v>
       </c>
     </row>
@@ -482,7 +542,12 @@
           <t>Barbados</t>
         </is>
       </c>
-      <c r="B13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BRB</t>
+        </is>
+      </c>
+      <c r="C13">
         <v>0.520311810771271</v>
       </c>
     </row>
@@ -492,7 +557,12 @@
           <t>Belarus</t>
         </is>
       </c>
-      <c r="B14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BLR</t>
+        </is>
+      </c>
+      <c r="C14">
         <v>0.1597832784982162</v>
       </c>
     </row>
@@ -502,7 +572,12 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="C15">
         <v>1</v>
       </c>
     </row>
@@ -512,7 +587,12 @@
           <t>Belize</t>
         </is>
       </c>
-      <c r="B16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BLZ</t>
+        </is>
+      </c>
+      <c r="C16">
         <v>0.798536461057017</v>
       </c>
     </row>
@@ -522,7 +602,12 @@
           <t>Benin</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BEN</t>
+        </is>
+      </c>
+      <c r="C17">
         <v>0.1436904086084926</v>
       </c>
     </row>
@@ -532,7 +617,12 @@
           <t>Bhutan</t>
         </is>
       </c>
-      <c r="B18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BTN</t>
+        </is>
+      </c>
+      <c r="C18">
         <v>1</v>
       </c>
     </row>
@@ -542,7 +632,12 @@
           <t>Bolivia (Plurinational State of)</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BOL</t>
+        </is>
+      </c>
+      <c r="C19">
         <v>0.2118610127392657</v>
       </c>
     </row>
@@ -552,7 +647,12 @@
           <t>Bosnia Herzegovina</t>
         </is>
       </c>
-      <c r="B20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BIH</t>
+        </is>
+      </c>
+      <c r="C20">
         <v>0.303092872921657</v>
       </c>
     </row>
@@ -562,7 +662,12 @@
           <t>Botswana</t>
         </is>
       </c>
-      <c r="B21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BWA</t>
+        </is>
+      </c>
+      <c r="C21">
         <v>0.3587457597156325</v>
       </c>
     </row>
@@ -572,7 +677,12 @@
           <t>Brazil</t>
         </is>
       </c>
-      <c r="B22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BRA</t>
+        </is>
+      </c>
+      <c r="C22">
         <v>0.2914401678082121</v>
       </c>
     </row>
@@ -582,7 +692,12 @@
           <t>Brunei Darussalam</t>
         </is>
       </c>
-      <c r="B23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BRN</t>
+        </is>
+      </c>
+      <c r="C23">
         <v>1</v>
       </c>
     </row>
@@ -592,7 +707,12 @@
           <t>Bulgaria</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BGR</t>
+        </is>
+      </c>
+      <c r="C24">
         <v>0.3594695890462891</v>
       </c>
     </row>
@@ -602,7 +722,12 @@
           <t>Burkina Faso</t>
         </is>
       </c>
-      <c r="B25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BFA</t>
+        </is>
+      </c>
+      <c r="C25">
         <v>1</v>
       </c>
     </row>
@@ -612,7 +737,12 @@
           <t>Burundi</t>
         </is>
       </c>
-      <c r="B26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BDI</t>
+        </is>
+      </c>
+      <c r="C26">
         <v>0.2201447819504314</v>
       </c>
     </row>
@@ -622,7 +752,12 @@
           <t>CÃ´te d'Ivoire</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CIV</t>
+        </is>
+      </c>
+      <c r="C27">
         <v>0.4167782884220189</v>
       </c>
     </row>
@@ -632,7 +767,12 @@
           <t>Cabo Verde</t>
         </is>
       </c>
-      <c r="B28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="C28">
         <v>0.3174019068094266</v>
       </c>
     </row>
@@ -642,7 +782,12 @@
           <t>Cambodia</t>
         </is>
       </c>
-      <c r="B29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>KHM</t>
+        </is>
+      </c>
+      <c r="C29">
         <v>1</v>
       </c>
     </row>
@@ -652,7 +797,12 @@
           <t>Cameroon</t>
         </is>
       </c>
-      <c r="B30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CMR</t>
+        </is>
+      </c>
+      <c r="C30">
         <v>0.2807818644772886</v>
       </c>
     </row>
@@ -662,7 +812,12 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="B31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="C31">
         <v>1</v>
       </c>
     </row>
@@ -672,7 +827,12 @@
           <t>Central African Rep.</t>
         </is>
       </c>
-      <c r="B32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CAF</t>
+        </is>
+      </c>
+      <c r="C32">
         <v>0.2981584268288978</v>
       </c>
     </row>
@@ -682,7 +842,12 @@
           <t>Chad</t>
         </is>
       </c>
-      <c r="B33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TCD</t>
+        </is>
+      </c>
+      <c r="C33">
         <v>0.3164406640419116</v>
       </c>
     </row>
@@ -692,7 +857,12 @@
           <t>Chile</t>
         </is>
       </c>
-      <c r="B34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>CHL</t>
+        </is>
+      </c>
+      <c r="C34">
         <v>0.6758929057012986</v>
       </c>
     </row>
@@ -702,7 +872,12 @@
           <t>China</t>
         </is>
       </c>
-      <c r="B35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CHN</t>
+        </is>
+      </c>
+      <c r="C35">
         <v>1</v>
       </c>
     </row>
@@ -712,7 +887,12 @@
           <t>China, Hong Kong SAR</t>
         </is>
       </c>
-      <c r="B36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HKG</t>
+        </is>
+      </c>
+      <c r="C36">
         <v>1</v>
       </c>
     </row>
@@ -722,7 +902,12 @@
           <t>China, Macao SAR</t>
         </is>
       </c>
-      <c r="B37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="C37">
         <v>1</v>
       </c>
     </row>
@@ -732,7 +917,12 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C38">
         <v>0.2014056710906114</v>
       </c>
     </row>
@@ -742,7 +932,12 @@
           <t>Comoros</t>
         </is>
       </c>
-      <c r="B39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C39">
         <v>0.5482296471546283</v>
       </c>
     </row>
@@ -752,7 +947,12 @@
           <t>Congo</t>
         </is>
       </c>
-      <c r="B40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>COG</t>
+        </is>
+      </c>
+      <c r="C40">
         <v>1</v>
       </c>
     </row>
@@ -762,7 +962,12 @@
           <t>Costa Rica</t>
         </is>
       </c>
-      <c r="B41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>CRI</t>
+        </is>
+      </c>
+      <c r="C41">
         <v>1</v>
       </c>
     </row>
@@ -772,7 +977,12 @@
           <t>Croatia</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HRV</t>
+        </is>
+      </c>
+      <c r="C42">
         <v>0.3305239049967512</v>
       </c>
     </row>
@@ -782,7 +992,12 @@
           <t>Cyprus</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CYP</t>
+        </is>
+      </c>
+      <c r="C43">
         <v>0.2800236908266892</v>
       </c>
     </row>
@@ -792,7 +1007,12 @@
           <t>Czechia</t>
         </is>
       </c>
-      <c r="B44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CZE</t>
+        </is>
+      </c>
+      <c r="C44">
         <v>1</v>
       </c>
     </row>
@@ -802,7 +1022,12 @@
           <t>Dem. People's Rep. of Korea</t>
         </is>
       </c>
-      <c r="B45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>PRK</t>
+        </is>
+      </c>
+      <c r="C45">
         <v>0.2215323264434766</v>
       </c>
     </row>
@@ -812,7 +1037,12 @@
           <t>Dem. Rep. of the Congo</t>
         </is>
       </c>
-      <c r="B46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="C46">
         <v>1</v>
       </c>
     </row>
@@ -822,7 +1052,12 @@
           <t>Denmark</t>
         </is>
       </c>
-      <c r="B47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DNK</t>
+        </is>
+      </c>
+      <c r="C47">
         <v>0.6203999760223021</v>
       </c>
     </row>
@@ -832,7 +1067,12 @@
           <t>Dominican Rep.</t>
         </is>
       </c>
-      <c r="B48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DOM</t>
+        </is>
+      </c>
+      <c r="C48">
         <v>0.4194529779802852</v>
       </c>
     </row>
@@ -842,7 +1082,12 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="B49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ECU</t>
+        </is>
+      </c>
+      <c r="C49">
         <v>0.4984714710931342</v>
       </c>
     </row>
@@ -852,7 +1097,12 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="B50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>EGY</t>
+        </is>
+      </c>
+      <c r="C50">
         <v>0.1228355213150182</v>
       </c>
     </row>
@@ -862,7 +1112,12 @@
           <t>El Salvador</t>
         </is>
       </c>
-      <c r="B51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SLV</t>
+        </is>
+      </c>
+      <c r="C51">
         <v>0.5652055409469136</v>
       </c>
     </row>
@@ -872,7 +1127,12 @@
           <t>Equatorial Guinea</t>
         </is>
       </c>
-      <c r="B52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>GNQ</t>
+        </is>
+      </c>
+      <c r="C52">
         <v>0.3916475479492498</v>
       </c>
     </row>
@@ -882,7 +1142,12 @@
           <t>Eritrea</t>
         </is>
       </c>
-      <c r="B53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ERI</t>
+        </is>
+      </c>
+      <c r="C53">
         <v>1</v>
       </c>
     </row>
@@ -892,7 +1157,12 @@
           <t>Estonia</t>
         </is>
       </c>
-      <c r="B54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="C54">
         <v>0.5101207499837994</v>
       </c>
     </row>
@@ -902,7 +1172,12 @@
           <t>Eswatini</t>
         </is>
       </c>
-      <c r="B55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SWZ</t>
+        </is>
+      </c>
+      <c r="C55">
         <v>1</v>
       </c>
     </row>
@@ -912,7 +1187,12 @@
           <t>Ethiopia</t>
         </is>
       </c>
-      <c r="B56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C56">
         <v>0.0417843186086336</v>
       </c>
     </row>
@@ -922,7 +1202,12 @@
           <t>Fiji</t>
         </is>
       </c>
-      <c r="B57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>FJI</t>
+        </is>
+      </c>
+      <c r="C57">
         <v>0.5587997367570332</v>
       </c>
     </row>
@@ -932,7 +1217,12 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="B58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>FIN</t>
+        </is>
+      </c>
+      <c r="C58">
         <v>0.4559846434769244</v>
       </c>
     </row>
@@ -942,7 +1232,12 @@
           <t>France</t>
         </is>
       </c>
-      <c r="B59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="C59">
         <v>0.547435917537278</v>
       </c>
     </row>
@@ -952,7 +1247,12 @@
           <t>French Polynesia</t>
         </is>
       </c>
-      <c r="B60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PYF</t>
+        </is>
+      </c>
+      <c r="C60">
         <v>0.5683322894909175</v>
       </c>
     </row>
@@ -962,7 +1262,12 @@
           <t>Gabon</t>
         </is>
       </c>
-      <c r="B61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>GAB</t>
+        </is>
+      </c>
+      <c r="C61">
         <v>0.8127430885657526</v>
       </c>
     </row>
@@ -972,7 +1277,12 @@
           <t>Gambia</t>
         </is>
       </c>
-      <c r="B62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>GMB</t>
+        </is>
+      </c>
+      <c r="C62">
         <v>0.4087798758669855</v>
       </c>
     </row>
@@ -982,7 +1292,12 @@
           <t>Georgia</t>
         </is>
       </c>
-      <c r="B63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>GEO</t>
+        </is>
+      </c>
+      <c r="C63">
         <v>0.1758416445214401</v>
       </c>
     </row>
@@ -992,7 +1307,12 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="B64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="C64">
         <v>1</v>
       </c>
     </row>
@@ -1002,7 +1322,12 @@
           <t>Ghana</t>
         </is>
       </c>
-      <c r="B65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>GHA</t>
+        </is>
+      </c>
+      <c r="C65">
         <v>0.2901082199863895</v>
       </c>
     </row>
@@ -1012,7 +1337,12 @@
           <t>Greece</t>
         </is>
       </c>
-      <c r="B66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>GRC</t>
+        </is>
+      </c>
+      <c r="C66">
         <v>0.277630146893028</v>
       </c>
     </row>
@@ -1022,7 +1352,12 @@
           <t>Guatemala</t>
         </is>
       </c>
-      <c r="B67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>GTM</t>
+        </is>
+      </c>
+      <c r="C67">
         <v>0.4646169068245586</v>
       </c>
     </row>
@@ -1032,7 +1367,12 @@
           <t>Guinea</t>
         </is>
       </c>
-      <c r="B68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>GIN</t>
+        </is>
+      </c>
+      <c r="C68">
         <v>1</v>
       </c>
     </row>
@@ -1042,7 +1382,12 @@
           <t>Guinea-Bissau</t>
         </is>
       </c>
-      <c r="B69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>GNB</t>
+        </is>
+      </c>
+      <c r="C69">
         <v>1</v>
       </c>
     </row>
@@ -1052,7 +1397,12 @@
           <t>Guyana</t>
         </is>
       </c>
-      <c r="B70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>GUY</t>
+        </is>
+      </c>
+      <c r="C70">
         <v>1</v>
       </c>
     </row>
@@ -1062,7 +1412,12 @@
           <t>Haiti</t>
         </is>
       </c>
-      <c r="B71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>HTI</t>
+        </is>
+      </c>
+      <c r="C71">
         <v>0.4173166285833901</v>
       </c>
     </row>
@@ -1072,7 +1427,12 @@
           <t>Honduras</t>
         </is>
       </c>
-      <c r="B72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>HND</t>
+        </is>
+      </c>
+      <c r="C72">
         <v>0.6942128187245068</v>
       </c>
     </row>
@@ -1082,7 +1442,12 @@
           <t>Hungary</t>
         </is>
       </c>
-      <c r="B73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>HUN</t>
+        </is>
+      </c>
+      <c r="C73">
         <v>1</v>
       </c>
     </row>
@@ -1092,7 +1457,12 @@
           <t>Iceland</t>
         </is>
       </c>
-      <c r="B74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ISL</t>
+        </is>
+      </c>
+      <c r="C74">
         <v>1</v>
       </c>
     </row>
@@ -1102,7 +1472,12 @@
           <t>India</t>
         </is>
       </c>
-      <c r="B75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="C75">
         <v>0.1668206646637334</v>
       </c>
     </row>
@@ -1112,7 +1487,12 @@
           <t>Indonesia</t>
         </is>
       </c>
-      <c r="B76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>IDN</t>
+        </is>
+      </c>
+      <c r="C76">
         <v>0.3126396737289734</v>
       </c>
     </row>
@@ -1122,7 +1502,12 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="B77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>IRN</t>
+        </is>
+      </c>
+      <c r="C77">
         <v>0.06305289870386077</v>
       </c>
     </row>
@@ -1132,7 +1517,12 @@
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>IRL</t>
+        </is>
+      </c>
+      <c r="C78">
         <v>1</v>
       </c>
     </row>
@@ -1142,7 +1532,12 @@
           <t>Israel</t>
         </is>
       </c>
-      <c r="B79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ISR</t>
+        </is>
+      </c>
+      <c r="C79">
         <v>0.4382649612795285</v>
       </c>
     </row>
@@ -1152,7 +1547,12 @@
           <t>Italy</t>
         </is>
       </c>
-      <c r="B80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="C80">
         <v>0.7948996144156466</v>
       </c>
     </row>
@@ -1162,7 +1562,12 @@
           <t>Jamaica</t>
         </is>
       </c>
-      <c r="B81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>JAM</t>
+        </is>
+      </c>
+      <c r="C81">
         <v>0.2213891821774714</v>
       </c>
     </row>
@@ -1172,7 +1577,12 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="B82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>JPN</t>
+        </is>
+      </c>
+      <c r="C82">
         <v>1</v>
       </c>
     </row>
@@ -1182,7 +1592,12 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="B83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>JOR</t>
+        </is>
+      </c>
+      <c r="C83">
         <v>0.3635042876428267</v>
       </c>
     </row>
@@ -1192,7 +1607,12 @@
           <t>Kazakhstan</t>
         </is>
       </c>
-      <c r="B84">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>KAZ</t>
+        </is>
+      </c>
+      <c r="C84">
         <v>0.2396092347032382</v>
       </c>
     </row>
@@ -1202,7 +1622,12 @@
           <t>Kenya</t>
         </is>
       </c>
-      <c r="B85">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>KEN</t>
+        </is>
+      </c>
+      <c r="C85">
         <v>0.1691527623854609</v>
       </c>
     </row>
@@ -1212,7 +1637,12 @@
           <t>Kuwait</t>
         </is>
       </c>
-      <c r="B86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>KWT</t>
+        </is>
+      </c>
+      <c r="C86">
         <v>1</v>
       </c>
     </row>
@@ -1222,7 +1652,12 @@
           <t>Kyrgyzstan</t>
         </is>
       </c>
-      <c r="B87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>KGZ</t>
+        </is>
+      </c>
+      <c r="C87">
         <v>1</v>
       </c>
     </row>
@@ -1232,7 +1667,12 @@
           <t>Lao People's Dem. Rep.</t>
         </is>
       </c>
-      <c r="B88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>LAO</t>
+        </is>
+      </c>
+      <c r="C88">
         <v>1</v>
       </c>
     </row>
@@ -1242,7 +1682,12 @@
           <t>Latvia</t>
         </is>
       </c>
-      <c r="B89">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>LVA</t>
+        </is>
+      </c>
+      <c r="C89">
         <v>0.5314365279843115</v>
       </c>
     </row>
@@ -1252,7 +1697,12 @@
           <t>Lesotho</t>
         </is>
       </c>
-      <c r="B90">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>LSO</t>
+        </is>
+      </c>
+      <c r="C90">
         <v>1</v>
       </c>
     </row>
@@ -1262,7 +1712,12 @@
           <t>Liberia</t>
         </is>
       </c>
-      <c r="B91">
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>LBR</t>
+        </is>
+      </c>
+      <c r="C91">
         <v>1</v>
       </c>
     </row>
@@ -1272,7 +1727,12 @@
           <t>Libya</t>
         </is>
       </c>
-      <c r="B92">
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>LBY</t>
+        </is>
+      </c>
+      <c r="C92">
         <v>0.5354510958564127</v>
       </c>
     </row>
@@ -1282,7 +1742,12 @@
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>LTU</t>
+        </is>
+      </c>
+      <c r="C93">
         <v>0.5378956570638219</v>
       </c>
     </row>
@@ -1292,7 +1757,12 @@
           <t>Luxembourg</t>
         </is>
       </c>
-      <c r="B94">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>LUX</t>
+        </is>
+      </c>
+      <c r="C94">
         <v>0.5439326370238536</v>
       </c>
     </row>
@@ -1302,7 +1772,12 @@
           <t>Madagascar</t>
         </is>
       </c>
-      <c r="B95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>MDG</t>
+        </is>
+      </c>
+      <c r="C95">
         <v>0.269337644191926</v>
       </c>
     </row>
@@ -1312,7 +1787,12 @@
           <t>Malawi</t>
         </is>
       </c>
-      <c r="B96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MWI</t>
+        </is>
+      </c>
+      <c r="C96">
         <v>0.2207450407261796</v>
       </c>
     </row>
@@ -1322,7 +1802,12 @@
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B97">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>MYS</t>
+        </is>
+      </c>
+      <c r="C97">
         <v>1</v>
       </c>
     </row>
@@ -1332,7 +1817,12 @@
           <t>Maldives</t>
         </is>
       </c>
-      <c r="B98">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>MDV</t>
+        </is>
+      </c>
+      <c r="C98">
         <v>0.3940067151528337</v>
       </c>
     </row>
@@ -1342,7 +1832,12 @@
           <t>Mali</t>
         </is>
       </c>
-      <c r="B99">
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>MLI</t>
+        </is>
+      </c>
+      <c r="C99">
         <v>0.07874981981923804</v>
       </c>
     </row>
@@ -1352,7 +1847,12 @@
           <t>Malta</t>
         </is>
       </c>
-      <c r="B100">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>MLT</t>
+        </is>
+      </c>
+      <c r="C100">
         <v>1</v>
       </c>
     </row>
@@ -1362,7 +1862,12 @@
           <t>Mauritania</t>
         </is>
       </c>
-      <c r="B101">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>MRT</t>
+        </is>
+      </c>
+      <c r="C101">
         <v>0.485258948745616</v>
       </c>
     </row>
@@ -1372,7 +1877,12 @@
           <t>Mauritius</t>
         </is>
       </c>
-      <c r="B102">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MUS</t>
+        </is>
+      </c>
+      <c r="C102">
         <v>0.3317139827003411</v>
       </c>
     </row>
@@ -1382,7 +1892,12 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="B103">
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>MEX</t>
+        </is>
+      </c>
+      <c r="C103">
         <v>1</v>
       </c>
     </row>
@@ -1392,7 +1907,12 @@
           <t>Mongolia</t>
         </is>
       </c>
-      <c r="B104">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>MNG</t>
+        </is>
+      </c>
+      <c r="C104">
         <v>1</v>
       </c>
     </row>
@@ -1402,7 +1922,12 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="B105">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="C105">
         <v>0.3644389345602631</v>
       </c>
     </row>
@@ -1412,7 +1937,12 @@
           <t>Mozambique</t>
         </is>
       </c>
-      <c r="B106">
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>MOZ</t>
+        </is>
+      </c>
+      <c r="C106">
         <v>0.3151714171536981</v>
       </c>
     </row>
@@ -1422,7 +1952,12 @@
           <t>Myanmar</t>
         </is>
       </c>
-      <c r="B107">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MMR</t>
+        </is>
+      </c>
+      <c r="C107">
         <v>0.2913291685844089</v>
       </c>
     </row>
@@ -1432,7 +1967,12 @@
           <t>Namibia</t>
         </is>
       </c>
-      <c r="B108">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>NAM</t>
+        </is>
+      </c>
+      <c r="C108">
         <v>0.6456289734185253</v>
       </c>
     </row>
@@ -1442,7 +1982,12 @@
           <t>Nepal</t>
         </is>
       </c>
-      <c r="B109">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>NPL</t>
+        </is>
+      </c>
+      <c r="C109">
         <v>0.2498234750552962</v>
       </c>
     </row>
@@ -1452,7 +1997,12 @@
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="B110">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>NLD</t>
+        </is>
+      </c>
+      <c r="C110">
         <v>1</v>
       </c>
     </row>
@@ -1462,7 +2012,12 @@
           <t>New Caledonia</t>
         </is>
       </c>
-      <c r="B111">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>NCL</t>
+        </is>
+      </c>
+      <c r="C111">
         <v>1</v>
       </c>
     </row>
@@ -1472,7 +2027,12 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="B112">
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>NZL</t>
+        </is>
+      </c>
+      <c r="C112">
         <v>0.4158418896605627</v>
       </c>
     </row>
@@ -1482,7 +2042,12 @@
           <t>Nicaragua</t>
         </is>
       </c>
-      <c r="B113">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>NIC</t>
+        </is>
+      </c>
+      <c r="C113">
         <v>1</v>
       </c>
     </row>
@@ -1492,7 +2057,12 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="B114">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>NER</t>
+        </is>
+      </c>
+      <c r="C114">
         <v>0.1396143494528409</v>
       </c>
     </row>
@@ -1502,7 +2072,12 @@
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="B115">
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>NGA</t>
+        </is>
+      </c>
+      <c r="C115">
         <v>0.1973121664968595</v>
       </c>
     </row>
@@ -1512,7 +2087,12 @@
           <t>North Macedonia</t>
         </is>
       </c>
-      <c r="B116">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>MKD</t>
+        </is>
+      </c>
+      <c r="C116">
         <v>1</v>
       </c>
     </row>
@@ -1522,7 +2102,12 @@
           <t>Norway</t>
         </is>
       </c>
-      <c r="B117">
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>NOR</t>
+        </is>
+      </c>
+      <c r="C117">
         <v>1</v>
       </c>
     </row>
@@ -1532,7 +2117,12 @@
           <t>Oman</t>
         </is>
       </c>
-      <c r="B118">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>OMN</t>
+        </is>
+      </c>
+      <c r="C118">
         <v>1</v>
       </c>
     </row>
@@ -1542,7 +2132,12 @@
           <t>Pakistan</t>
         </is>
       </c>
-      <c r="B119">
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="C119">
         <v>0.208130613239764</v>
       </c>
     </row>
@@ -1552,7 +2147,12 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="B120">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C120">
         <v>0.4838338334128947</v>
       </c>
     </row>
@@ -1562,7 +2162,12 @@
           <t>Papua New Guinea</t>
         </is>
       </c>
-      <c r="B121">
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="C121">
         <v>1</v>
       </c>
     </row>
@@ -1572,7 +2177,12 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="B122">
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>PRY</t>
+        </is>
+      </c>
+      <c r="C122">
         <v>0.5364685825085852</v>
       </c>
     </row>
@@ -1582,7 +2192,12 @@
           <t>Peru</t>
         </is>
       </c>
-      <c r="B123">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="C123">
         <v>0.503337744593336</v>
       </c>
     </row>
@@ -1592,7 +2207,12 @@
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B124">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>PHL</t>
+        </is>
+      </c>
+      <c r="C124">
         <v>0.3884208878455885</v>
       </c>
     </row>
@@ -1602,7 +2222,12 @@
           <t>Poland</t>
         </is>
       </c>
-      <c r="B125">
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>POL</t>
+        </is>
+      </c>
+      <c r="C125">
         <v>0.6805697508052662</v>
       </c>
     </row>
@@ -1612,7 +2237,12 @@
           <t>Portugal</t>
         </is>
       </c>
-      <c r="B126">
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="C126">
         <v>0.3618374994872768</v>
       </c>
     </row>
@@ -1622,7 +2252,12 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="B127">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>QAT</t>
+        </is>
+      </c>
+      <c r="C127">
         <v>1</v>
       </c>
     </row>
@@ -1632,7 +2267,12 @@
           <t>Rep. of Korea</t>
         </is>
       </c>
-      <c r="B128">
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>KOR</t>
+        </is>
+      </c>
+      <c r="C128">
         <v>1</v>
       </c>
     </row>
@@ -1642,7 +2282,12 @@
           <t>Rep. of Moldova</t>
         </is>
       </c>
-      <c r="B129">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>MDA</t>
+        </is>
+      </c>
+      <c r="C129">
         <v>0.3757666943819667</v>
       </c>
     </row>
@@ -1652,7 +2297,12 @@
           <t>Romania</t>
         </is>
       </c>
-      <c r="B130">
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>ROU</t>
+        </is>
+      </c>
+      <c r="C130">
         <v>0.3793414347258627</v>
       </c>
     </row>
@@ -1662,7 +2312,12 @@
           <t>Russian Federation</t>
         </is>
       </c>
-      <c r="B131">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>RUS</t>
+        </is>
+      </c>
+      <c r="C131">
         <v>1</v>
       </c>
     </row>
@@ -1672,7 +2327,12 @@
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="B132">
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>RWA</t>
+        </is>
+      </c>
+      <c r="C132">
         <v>0.120828982255026</v>
       </c>
     </row>
@@ -1682,7 +2342,12 @@
           <t>Saint Lucia</t>
         </is>
       </c>
-      <c r="B133">
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>LCA</t>
+        </is>
+      </c>
+      <c r="C133">
         <v>1</v>
       </c>
     </row>
@@ -1692,7 +2357,12 @@
           <t>Saint Vincent and the Grenadines</t>
         </is>
       </c>
-      <c r="B134">
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>VCT</t>
+        </is>
+      </c>
+      <c r="C134">
         <v>1</v>
       </c>
     </row>
@@ -1702,7 +2372,12 @@
           <t>Samoa</t>
         </is>
       </c>
-      <c r="B135">
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>WSM</t>
+        </is>
+      </c>
+      <c r="C135">
         <v>0.6722419393375387</v>
       </c>
     </row>
@@ -1712,7 +2387,12 @@
           <t>Sao Tome and Principe</t>
         </is>
       </c>
-      <c r="B136">
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>STP</t>
+        </is>
+      </c>
+      <c r="C136">
         <v>1</v>
       </c>
     </row>
@@ -1722,7 +2402,12 @@
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="B137">
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SAU</t>
+        </is>
+      </c>
+      <c r="C137">
         <v>0.4434388439114125</v>
       </c>
     </row>
@@ -1732,7 +2417,12 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="B138">
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>SEN</t>
+        </is>
+      </c>
+      <c r="C138">
         <v>0.2123155248610868</v>
       </c>
     </row>
@@ -1742,7 +2432,12 @@
           <t>Sierra Leone</t>
         </is>
       </c>
-      <c r="B139">
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>SLE</t>
+        </is>
+      </c>
+      <c r="C139">
         <v>0.5310322093271261</v>
       </c>
     </row>
@@ -1752,7 +2447,12 @@
           <t>Singapore</t>
         </is>
       </c>
-      <c r="B140">
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>SGP</t>
+        </is>
+      </c>
+      <c r="C140">
         <v>0.9999999999999999</v>
       </c>
     </row>
@@ -1762,7 +2462,12 @@
           <t>Slovakia</t>
         </is>
       </c>
-      <c r="B141">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>SVK</t>
+        </is>
+      </c>
+      <c r="C141">
         <v>1</v>
       </c>
     </row>
@@ -1772,7 +2477,12 @@
           <t>Slovenia</t>
         </is>
       </c>
-      <c r="B142">
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>SVN</t>
+        </is>
+      </c>
+      <c r="C142">
         <v>1</v>
       </c>
     </row>
@@ -1782,7 +2492,12 @@
           <t>Solomon Isds</t>
         </is>
       </c>
-      <c r="B143">
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C143">
         <v>1</v>
       </c>
     </row>
@@ -1792,7 +2507,12 @@
           <t>Somalia</t>
         </is>
       </c>
-      <c r="B144">
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SOM</t>
+        </is>
+      </c>
+      <c r="C144">
         <v>0.1413604713340993</v>
       </c>
     </row>
@@ -1802,7 +2522,12 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="B145">
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>ZAF</t>
+        </is>
+      </c>
+      <c r="C145">
         <v>0.4218114323293546</v>
       </c>
     </row>
@@ -1812,7 +2537,12 @@
           <t>Spain</t>
         </is>
       </c>
-      <c r="B146">
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="C146">
         <v>0.401958603987669</v>
       </c>
     </row>
@@ -1822,7 +2552,12 @@
           <t>Sri Lanka</t>
         </is>
       </c>
-      <c r="B147">
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="C147">
         <v>0.323938012079828</v>
       </c>
     </row>
@@ -1832,7 +2567,12 @@
           <t>Suriname</t>
         </is>
       </c>
-      <c r="B148">
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SUR</t>
+        </is>
+      </c>
+      <c r="C148">
         <v>1</v>
       </c>
     </row>
@@ -1842,7 +2582,12 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="B149">
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>SWE</t>
+        </is>
+      </c>
+      <c r="C149">
         <v>0.5324564882752129</v>
       </c>
     </row>
@@ -1852,7 +2597,12 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="B150">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>CHE</t>
+        </is>
+      </c>
+      <c r="C150">
         <v>1</v>
       </c>
     </row>
@@ -1862,7 +2612,12 @@
           <t>Syria</t>
         </is>
       </c>
-      <c r="B151">
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>SYR</t>
+        </is>
+      </c>
+      <c r="C151">
         <v>0.05969165777875399</v>
       </c>
     </row>
@@ -1872,7 +2627,12 @@
           <t>TÃ¼rkiye</t>
         </is>
       </c>
-      <c r="B152">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>TUR</t>
+        </is>
+      </c>
+      <c r="C152">
         <v>0.4048317361377607</v>
       </c>
     </row>
@@ -1882,7 +2642,12 @@
           <t>Tajikistan</t>
         </is>
       </c>
-      <c r="B153">
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>TJK</t>
+        </is>
+      </c>
+      <c r="C153">
         <v>0.248406628357956</v>
       </c>
     </row>
@@ -1892,7 +2657,12 @@
           <t>Thailand</t>
         </is>
       </c>
-      <c r="B154">
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="C154">
         <v>0.6400577145294765</v>
       </c>
     </row>
@@ -1902,7 +2672,12 @@
           <t>Timor-Leste</t>
         </is>
       </c>
-      <c r="B155">
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
+      <c r="C155">
         <v>0.3524545824459783</v>
       </c>
     </row>
@@ -1912,7 +2687,12 @@
           <t>Togo</t>
         </is>
       </c>
-      <c r="B156">
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>TGO</t>
+        </is>
+      </c>
+      <c r="C156">
         <v>1</v>
       </c>
     </row>
@@ -1922,7 +2702,12 @@
           <t>Tonga</t>
         </is>
       </c>
-      <c r="B157">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>TON</t>
+        </is>
+      </c>
+      <c r="C157">
         <v>1</v>
       </c>
     </row>
@@ -1932,7 +2717,12 @@
           <t>Trinidad and Tobago</t>
         </is>
       </c>
-      <c r="B158">
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>TTO</t>
+        </is>
+      </c>
+      <c r="C158">
         <v>1</v>
       </c>
     </row>
@@ -1942,7 +2732,12 @@
           <t>Tunisia</t>
         </is>
       </c>
-      <c r="B159">
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>TUN</t>
+        </is>
+      </c>
+      <c r="C159">
         <v>0.3638443243035466</v>
       </c>
     </row>
@@ -1952,7 +2747,12 @@
           <t>Turkmenistan</t>
         </is>
       </c>
-      <c r="B160">
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>TKM</t>
+        </is>
+      </c>
+      <c r="C160">
         <v>0.4323575536668961</v>
       </c>
     </row>
@@ -1962,7 +2762,12 @@
           <t>Uganda</t>
         </is>
       </c>
-      <c r="B161">
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>UGA</t>
+        </is>
+      </c>
+      <c r="C161">
         <v>0.3043801091450877</v>
       </c>
     </row>
@@ -1972,7 +2777,12 @@
           <t>United Arab Emirates</t>
         </is>
       </c>
-      <c r="B162">
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>ARE</t>
+        </is>
+      </c>
+      <c r="C162">
         <v>1</v>
       </c>
     </row>
@@ -1982,7 +2792,12 @@
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B163">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="C163">
         <v>0.3553073170027465</v>
       </c>
     </row>
@@ -1992,7 +2807,12 @@
           <t>United Rep. of Tanzania</t>
         </is>
       </c>
-      <c r="B164">
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>TZA</t>
+        </is>
+      </c>
+      <c r="C164">
         <v>0.200438941800422</v>
       </c>
     </row>
@@ -2002,7 +2822,12 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B165">
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>URY</t>
+        </is>
+      </c>
+      <c r="C165">
         <v>0.324537095646835</v>
       </c>
     </row>
@@ -2012,7 +2837,12 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="B166">
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C166">
         <v>1</v>
       </c>
     </row>
@@ -2022,7 +2852,12 @@
           <t>Uzbekistan</t>
         </is>
       </c>
-      <c r="B167">
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>UZB</t>
+        </is>
+      </c>
+      <c r="C167">
         <v>0.2746748871548846</v>
       </c>
     </row>
@@ -2032,7 +2867,12 @@
           <t>Vanuatu</t>
         </is>
       </c>
-      <c r="B168">
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>VUT</t>
+        </is>
+      </c>
+      <c r="C168">
         <v>1</v>
       </c>
     </row>
@@ -2042,7 +2882,12 @@
           <t>Venezuela</t>
         </is>
       </c>
-      <c r="B169">
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>VEN</t>
+        </is>
+      </c>
+      <c r="C169">
         <v>0.2157141182899774</v>
       </c>
     </row>
@@ -2052,7 +2897,12 @@
           <t>Viet Nam</t>
         </is>
       </c>
-      <c r="B170">
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>VNM</t>
+        </is>
+      </c>
+      <c r="C170">
         <v>1</v>
       </c>
     </row>
@@ -2062,7 +2912,12 @@
           <t>Yemen</t>
         </is>
       </c>
-      <c r="B171">
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>YEM</t>
+        </is>
+      </c>
+      <c r="C171">
         <v>0.1914405009827123</v>
       </c>
     </row>
@@ -2072,7 +2927,12 @@
           <t>Zambia</t>
         </is>
       </c>
-      <c r="B172">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>ZMB</t>
+        </is>
+      </c>
+      <c r="C172">
         <v>0.5873648727189525</v>
       </c>
     </row>
@@ -2082,7 +2942,12 @@
           <t>Zimbabwe</t>
         </is>
       </c>
-      <c r="B173">
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="C173">
         <v>0.3992652556614511</v>
       </c>
     </row>

</xml_diff>